<commit_message>
Implement prompt regression metrics
</commit_message>
<xml_diff>
--- a/docs/IMPLEMENTED_JUDGE_METRICS.xlsx
+++ b/docs/IMPLEMENTED_JUDGE_METRICS.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implemented Metrics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Implemented Metrics'!$A$1:$I$12</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,22 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -57,14 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -445,549 +428,728 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Detector Method</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Trace Events Used</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Trace Fields Used</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Failure Rule</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>output_contract_compliance</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>critical/high</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Prompt / Instruction</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>output_contract()</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>final_output</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>final_output.content</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>final_output missing/empty or required markdown sections missing</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>0.95</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>target_endpoint_consistency</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Tool Use</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>wrong_endpoint()</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>run_start/chat_turn_start, tool_start, tool_end</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>user_input, filter_log_records.path_pattern, compute_log_metrics.top_paths[].path</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>tool argument or metric path differs from user target path</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>0.96</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>metric_result_consistency</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Final Output / Completion</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>metric_consistency()</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>react_step, tool_end, node_start, node_end</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>react_step.action, tool_end.tool, state.metrics.faultInjected</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>compute step without compute_log_metrics result or faultInjected metrics</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>0.90/0.98</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>validation_path_coverage</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>LangGraph Flow</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>validation_path()</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>node_start, validation_result, edge_selected</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>node_start.node, validation_result count, edge_selected.reason</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>validate_findings node/result missing or validation skip edge detected</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>0.98</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>parse_error_handling_score</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Tool Use</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>parse_error_handling()</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>tool_end(parse_access_log), final_output, validation_result</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>parse_error_count, total_lines, final_output.content, validation_result.issues</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>parse_error_count / total_lines &gt; 0.5</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>0.94</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>rag_context_presence_and_usage</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Context / Retrieval</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>rag_mcp_presence()</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>tool_end, final_output</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>tool_end.tool, final_output.content</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>retrieve_runbook missing or ## RAG Context missing</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>0.85/0.80</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>instruction_adherence_score</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Prompt / Instruction</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>instruction_adherence()</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>prompt_instruction_metrics</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>instruction_adherence.score, instruction_adherence.violations</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>score &lt; 1.0 or violations present</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>0.90</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>mcp_context_presence_and_usage</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>ReAct / RAG / MCP</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>rag_mcp_presence()</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>mcp_end, final_output</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>mcp_end.method, final_output.content</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>mcp tools/call missing or ## MCP Context missing</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>0.85/0.80</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>chat_context_grounding</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>medium/low</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Context / Retrieval</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>chat_context()</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>chat_*, chat_analysis_invoked, chat_context_built, chat_response_generated</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>chat_context_built.has_last_analysis</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>follow-up response not grounded in last analysis/context evidence</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>0.82/0.70</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>output_format_compliance</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Prompt / Instruction</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>output_format_compliance()</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>prompt_instruction_metrics, final_output fallback</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>output_format.compliant, output_format.missing_sections</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>required output format is not compliant</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>0.92</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>prompt_template_version_present</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Prompt / Instruction</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>prompt_template_version()</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>instruction_snapshot, prompt_instruction_metrics</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>prompt_template.name, prompt_template.version, prompt_template.present</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>prompt template name/version missing</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>0.90</t>
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>prompt_version_regression_score</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>critical/high</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Prompt / Instruction</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>detect_prompt_regressions()</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>baseline/candidate AnalysisResult</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>baseline.score, candidate.score, gate delta, new findings</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>regression score &lt; 85</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>gate_regression</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>critical/high</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Prompt / Instruction</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>detect_prompt_regressions()</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>baseline/candidate AnalysisResult</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>baseline.gate, candidate.gate</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>candidate gate rank &gt; baseline gate rank</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>new_high_severity_findings</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>critical/high</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Prompt / Instruction</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>detect_prompt_regressions()</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>baseline/candidate findings</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>finding metric/category/location/evidence diff</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>candidate introduces new high/critical findings</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>tool_and_output_stability_score</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>medium/high</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Prompt / Instruction</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>detect_prompt_regressions()</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>baseline/candidate trace events</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>tool_start sequence, validation path, output compliance, target endpoint findings</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>stability score &lt; 0.85</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0.86</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>